<commit_message>
update KL/FM to column A before total
</commit_message>
<xml_diff>
--- a/FMBrandFY2026FebRollingCost20260420_copy.xlsx
+++ b/FMBrandFY2026FebRollingCost20260420_copy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shenkailing\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{12B4572D-4090-4C58-9077-DCF6EA27FB1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F7F89618-E8B3-443B-B0FD-B5DBB2C038DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{50365140-748A-4C84-BBCE-58A45EFCD935}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{6D11DB6E-EB7E-45F0-BEAE-6BAD57BFB6B5}"/>
   </bookViews>
   <sheets>
     <sheet name="CostCenterGroupBySumResult" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="178">
   <si>
     <t>品牌</t>
   </si>
@@ -356,166 +356,170 @@
     <t>调整后福利合计</t>
   </si>
   <si>
+    <t>KL/FM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FY2026</t>
+  </si>
+  <si>
+    <t>杭州</t>
+  </si>
+  <si>
+    <t>杭州银泰</t>
+  </si>
+  <si>
+    <t>BA</t>
+  </si>
+  <si>
+    <t>KLFMFY2021000003</t>
+  </si>
+  <si>
+    <t>Existing</t>
+  </si>
+  <si>
+    <t>DS</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Tier I cities</t>
+  </si>
+  <si>
+    <t>北京</t>
+  </si>
+  <si>
+    <t>北京新光三越</t>
+  </si>
+  <si>
+    <t>KLFMFY2021000002</t>
+  </si>
+  <si>
+    <t>IN77银泰</t>
+  </si>
+  <si>
+    <t>KLFMFY2021000004</t>
+  </si>
+  <si>
+    <t>宁波</t>
+  </si>
+  <si>
+    <t>宁波阪急-498</t>
+  </si>
+  <si>
+    <t>KLFMFY2023000026</t>
+  </si>
+  <si>
+    <t>Tier II cities +</t>
+  </si>
+  <si>
+    <t>杭州万象城</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>KLFMFY2022000013</t>
+  </si>
+  <si>
+    <t>FSS</t>
+  </si>
+  <si>
+    <t>成都</t>
+  </si>
+  <si>
+    <t>成都远洋太古里</t>
+  </si>
+  <si>
+    <t>KLFMFY2023000025</t>
+  </si>
+  <si>
+    <t>成都SKP</t>
+  </si>
+  <si>
+    <t>KLFMFY2023000024</t>
+  </si>
+  <si>
+    <t>武汉</t>
+  </si>
+  <si>
+    <t>武汉SKP</t>
+  </si>
+  <si>
+    <t>KLFMFY2023000023</t>
+  </si>
+  <si>
+    <t>重庆</t>
+  </si>
+  <si>
+    <t>重庆星光68</t>
+  </si>
+  <si>
+    <t>KLFMFY2024000012</t>
+  </si>
+  <si>
+    <t>深圳</t>
+  </si>
+  <si>
+    <t>深圳万象天地</t>
+  </si>
+  <si>
+    <t>KLFMFY2022000011</t>
+  </si>
+  <si>
+    <t>南京</t>
+  </si>
+  <si>
+    <t>南京德基</t>
+  </si>
+  <si>
+    <t>KLFMFY2022000010</t>
+  </si>
+  <si>
+    <t>深圳罗湖万象城</t>
+  </si>
+  <si>
+    <t>KLFMFY2022000012</t>
+  </si>
+  <si>
+    <t>北京三里屯</t>
+  </si>
+  <si>
+    <t>KLFMFY2022000016</t>
+  </si>
+  <si>
+    <t>上海</t>
+  </si>
+  <si>
+    <t>上海前滩太古里</t>
+  </si>
+  <si>
+    <t>KLFMFY2022000015</t>
+  </si>
+  <si>
+    <t>contingency 柜台</t>
+  </si>
+  <si>
+    <t>KLFMFY2022000014</t>
+  </si>
+  <si>
+    <t>Contingency</t>
+  </si>
+  <si>
+    <t>FY2026 新店3</t>
+  </si>
+  <si>
+    <t>KLFMFY2026000003</t>
+  </si>
+  <si>
+    <t>FY26 New Door</t>
+  </si>
+  <si>
+    <t>Total:</t>
+  </si>
+  <si>
     <t>FM</t>
-  </si>
-  <si>
-    <t>FY2026</t>
-  </si>
-  <si>
-    <t>杭州</t>
-  </si>
-  <si>
-    <t>杭州银泰</t>
-  </si>
-  <si>
-    <t>BA</t>
-  </si>
-  <si>
-    <t>KLFMFY2021000003</t>
-  </si>
-  <si>
-    <t>Existing</t>
-  </si>
-  <si>
-    <t>DS</t>
-  </si>
-  <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>Tier I cities</t>
-  </si>
-  <si>
-    <t>北京</t>
-  </si>
-  <si>
-    <t>北京新光三越</t>
-  </si>
-  <si>
-    <t>KLFMFY2021000002</t>
-  </si>
-  <si>
-    <t>IN77银泰</t>
-  </si>
-  <si>
-    <t>KLFMFY2021000004</t>
-  </si>
-  <si>
-    <t>宁波</t>
-  </si>
-  <si>
-    <t>宁波阪急-498</t>
-  </si>
-  <si>
-    <t>KLFMFY2023000026</t>
-  </si>
-  <si>
-    <t>Tier II cities +</t>
-  </si>
-  <si>
-    <t>杭州万象城</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>KLFMFY2022000013</t>
-  </si>
-  <si>
-    <t>FSS</t>
-  </si>
-  <si>
-    <t>成都</t>
-  </si>
-  <si>
-    <t>成都远洋太古里</t>
-  </si>
-  <si>
-    <t>KLFMFY2023000025</t>
-  </si>
-  <si>
-    <t>成都SKP</t>
-  </si>
-  <si>
-    <t>KLFMFY2023000024</t>
-  </si>
-  <si>
-    <t>武汉</t>
-  </si>
-  <si>
-    <t>武汉SKP</t>
-  </si>
-  <si>
-    <t>KLFMFY2023000023</t>
-  </si>
-  <si>
-    <t>重庆</t>
-  </si>
-  <si>
-    <t>重庆星光68</t>
-  </si>
-  <si>
-    <t>KLFMFY2024000012</t>
-  </si>
-  <si>
-    <t>深圳</t>
-  </si>
-  <si>
-    <t>深圳万象天地</t>
-  </si>
-  <si>
-    <t>KLFMFY2022000011</t>
-  </si>
-  <si>
-    <t>南京</t>
-  </si>
-  <si>
-    <t>南京德基</t>
-  </si>
-  <si>
-    <t>KLFMFY2022000010</t>
-  </si>
-  <si>
-    <t>深圳罗湖万象城</t>
-  </si>
-  <si>
-    <t>KLFMFY2022000012</t>
-  </si>
-  <si>
-    <t>北京三里屯</t>
-  </si>
-  <si>
-    <t>KLFMFY2022000016</t>
-  </si>
-  <si>
-    <t>上海</t>
-  </si>
-  <si>
-    <t>上海前滩太古里</t>
-  </si>
-  <si>
-    <t>KLFMFY2022000015</t>
-  </si>
-  <si>
-    <t>contingency 柜台</t>
-  </si>
-  <si>
-    <t>KLFMFY2022000014</t>
-  </si>
-  <si>
-    <t>Contingency</t>
-  </si>
-  <si>
-    <t>FY2026 新店3</t>
-  </si>
-  <si>
-    <t>KLFMFY2026000003</t>
-  </si>
-  <si>
-    <t>FY26 New Door</t>
-  </si>
-  <si>
-    <t>Total:</t>
   </si>
   <si>
     <t>上海国金中心</t>
@@ -571,10 +575,6 @@
   </si>
   <si>
     <t>FM Total:</t>
-  </si>
-  <si>
-    <t>TEST</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1012,9 +1012,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46945E5-4B62-4EC0-8E35-79E90B969C0E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{615F0CC5-9A04-405F-8E2E-99FD20546223}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:DA37"/>
+  <dimension ref="A1:DA33"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:105" x14ac:dyDescent="0.3">
@@ -7104,7 +7104,7 @@
     </row>
     <row r="21" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
-        <v>105</v>
+        <v>159</v>
       </c>
       <c r="B21" s="8" t="s">
         <v>106</v>
@@ -7113,7 +7113,7 @@
         <v>149</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E21" s="8" t="s">
         <v>125</v>
@@ -7128,10 +7128,10 @@
         <v>109</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K21" s="8" t="s">
         <v>111</v>
@@ -7417,20 +7417,20 @@
     </row>
     <row r="22" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>106</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G22" s="3">
         <v>5842263202</v>
@@ -7439,10 +7439,10 @@
         <v>109</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>157</v>
@@ -7726,7 +7726,7 @@
     </row>
     <row r="23" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>106</v>
@@ -7735,11 +7735,11 @@
         <v>107</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E23" s="8"/>
       <c r="F23" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G23" s="8">
         <v>5841813202</v>
@@ -7748,10 +7748,10 @@
         <v>109</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K23" s="8" t="s">
         <v>157</v>
@@ -8035,20 +8035,20 @@
     </row>
     <row r="24" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>106</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G24" s="3">
         <v>5842263202</v>
@@ -8057,10 +8057,10 @@
         <v>109</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K24" s="3" t="s">
         <v>157</v>
@@ -8344,7 +8344,7 @@
     </row>
     <row r="25" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>106</v>
@@ -8353,11 +8353,11 @@
         <v>107</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E25" s="8"/>
       <c r="F25" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G25" s="8">
         <v>5841813202</v>
@@ -8366,10 +8366,10 @@
         <v>109</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K25" s="8" t="s">
         <v>157</v>
@@ -8654,7 +8654,7 @@
     <row r="26" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
       <c r="B26" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
@@ -9136,16 +9136,16 @@
     </row>
     <row r="28" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>105</v>
+        <v>159</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>106</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>125</v>
@@ -9160,10 +9160,10 @@
         <v>109</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K28" s="3" t="s">
         <v>111</v>
@@ -9449,20 +9449,20 @@
     </row>
     <row r="29" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
-        <v>105</v>
+        <v>159</v>
       </c>
       <c r="B29" s="8" t="s">
         <v>106</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E29" s="8"/>
       <c r="F29" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G29" s="8">
         <v>5841813202</v>
@@ -9471,10 +9471,10 @@
         <v>109</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K29" s="8" t="s">
         <v>157</v>
@@ -9758,7 +9758,7 @@
     </row>
     <row r="30" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>105</v>
+        <v>159</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>106</v>
@@ -9767,11 +9767,11 @@
         <v>107</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E30" s="3"/>
       <c r="F30" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G30" s="3">
         <v>5841813202</v>
@@ -9780,10 +9780,10 @@
         <v>109</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K30" s="3" t="s">
         <v>157</v>
@@ -10067,7 +10067,7 @@
     </row>
     <row r="31" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
-        <v>105</v>
+        <v>159</v>
       </c>
       <c r="B31" s="8" t="s">
         <v>106</v>
@@ -10076,11 +10076,11 @@
         <v>107</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E31" s="8"/>
       <c r="F31" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G31" s="8">
         <v>5841813202</v>
@@ -10089,10 +10089,10 @@
         <v>109</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K31" s="8" t="s">
         <v>157</v>
@@ -10377,7 +10377,7 @@
     <row r="32" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
@@ -10750,7 +10750,7 @@
         <v>158000</v>
       </c>
     </row>
-    <row r="33" spans="1:105" x14ac:dyDescent="0.3">
+    <row r="33" spans="17:105" x14ac:dyDescent="0.3">
       <c r="Q33" s="12"/>
       <c r="R33" s="12"/>
       <c r="S33" s="12"/>
@@ -10841,50 +10841,6 @@
       <c r="CZ33" s="12"/>
       <c r="DA33" s="12"/>
     </row>
-    <row r="34" spans="1:105" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>177</v>
-      </c>
-      <c r="B34" t="s">
-        <v>177</v>
-      </c>
-      <c r="C34" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="35" spans="1:105" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>177</v>
-      </c>
-      <c r="B35" t="s">
-        <v>177</v>
-      </c>
-      <c r="C35" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="36" spans="1:105" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>177</v>
-      </c>
-      <c r="B36" t="s">
-        <v>177</v>
-      </c>
-      <c r="C36" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="37" spans="1:105" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>177</v>
-      </c>
-      <c r="B37" t="s">
-        <v>177</v>
-      </c>
-      <c r="C37" t="s">
-        <v>177</v>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update column c according column a and column b
</commit_message>
<xml_diff>
--- a/FMBrandFY2026FebRollingCost20260420_copy.xlsx
+++ b/FMBrandFY2026FebRollingCost20260420_copy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shenkailing\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F7F89618-E8B3-443B-B0FD-B5DBB2C038DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1FE2FE04-293E-41D7-AAE2-77A34EFBC7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{6D11DB6E-EB7E-45F0-BEAE-6BAD57BFB6B5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{6B65AC86-F445-43C6-AE3F-ABA7E8B83D93}"/>
   </bookViews>
   <sheets>
     <sheet name="CostCenterGroupBySumResult" sheetId="1" r:id="rId1"/>
@@ -519,19 +519,16 @@
     <t>Total:</t>
   </si>
   <si>
-    <t>FM</t>
-  </si>
-  <si>
-    <t>上海国金中心</t>
-  </si>
-  <si>
-    <t>KLFMFY2020000001</t>
-  </si>
-  <si>
     <t>KL</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>上海国金中心</t>
+  </si>
+  <si>
+    <t>KLFMFY2020000001</t>
+  </si>
+  <si>
     <t>苏州</t>
   </si>
   <si>
@@ -548,6 +545,10 @@
   </si>
   <si>
     <t>KL Total:</t>
+  </si>
+  <si>
+    <t>FM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>广州</t>
@@ -654,7 +655,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -677,8 +678,6 @@
     <xf numFmtId="4" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1012,8 +1011,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{615F0CC5-9A04-405F-8E2E-99FD20546223}">
-  <sheetPr codeName="Sheet3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD8C1425-B57F-4B09-902D-3BC8F75F9A54}">
+  <sheetPr codeName="Sheet18"/>
   <dimension ref="A1:DA33"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -6636,363 +6635,369 @@
       <c r="L19" s="8"/>
       <c r="M19" s="9"/>
       <c r="N19" s="9"/>
-      <c r="O19" s="10"/>
-      <c r="P19" s="10"/>
+      <c r="O19" s="10">
+        <f>SUM($O$3,$O$4,$O$5,$O$6,$O$7,$O$8,$O$9,$O$10,$O$11,$O$12,$O$13,$O$14,$O$15,$O$16,$O$17,$O$18)</f>
+        <v>0</v>
+      </c>
+      <c r="P19" s="10">
+        <f>SUM($P$3,$P$4,$P$5,$P$6,$P$7,$P$8,$P$9,$P$10,$P$11,$P$12,$P$13,$P$14,$P$15,$P$16,$P$17,$P$18)</f>
+        <v>0</v>
+      </c>
       <c r="Q19" s="11">
-        <f>SUM($Q$2,$Q$3,$Q$4,$Q$5,$Q$6,$Q$7,$Q$8,$Q$9,$Q$10,$Q$11,$Q$12,$Q$13,$Q$14,$Q$15,$Q$16,$Q$17,$Q$18)</f>
+        <f>SUM($Q$3,$Q$4,$Q$5,$Q$6,$Q$7,$Q$8,$Q$9,$Q$10,$Q$11,$Q$12,$Q$13,$Q$14,$Q$15,$Q$16,$Q$17,$Q$18)</f>
         <v>0</v>
       </c>
       <c r="R19" s="11">
-        <f>SUM($R$2,$R$3,$R$4,$R$5,$R$6,$R$7,$R$8,$R$9,$R$10,$R$11,$R$12,$R$13,$R$14,$R$15,$R$16,$R$17,$R$18)</f>
+        <f>SUM($R$3,$R$4,$R$5,$R$6,$R$7,$R$8,$R$9,$R$10,$R$11,$R$12,$R$13,$R$14,$R$15,$R$16,$R$17,$R$18)</f>
         <v>0</v>
       </c>
       <c r="S19" s="6">
-        <f>SUM($S$2,$S$3,$S$4,$S$5,$S$6,$S$7,$S$8,$S$9,$S$10,$S$11,$S$12,$S$13,$S$14,$S$15,$S$16,$S$17,$S$18)</f>
+        <f>SUM($S$3,$S$4,$S$5,$S$6,$S$7,$S$8,$S$9,$S$10,$S$11,$S$12,$S$13,$S$14,$S$15,$S$16,$S$17,$S$18)</f>
+        <v>64000</v>
+      </c>
+      <c r="T19" s="6">
+        <f>SUM($T$3,$T$4,$T$5,$T$6,$T$7,$T$8,$T$9,$T$10,$T$11,$T$12,$T$13,$T$14,$T$15,$T$16,$T$17,$T$18)</f>
+        <v>64000</v>
+      </c>
+      <c r="U19" s="11">
+        <f>SUM($U$3,$U$4,$U$5,$U$6,$U$7,$U$8,$U$9,$U$10,$U$11,$U$12,$U$13,$U$14,$U$15,$U$16,$U$17,$U$18)</f>
+        <v>64</v>
+      </c>
+      <c r="V19" s="11">
+        <f>SUM($V$3,$V$4,$V$5,$V$6,$V$7,$V$8,$V$9,$V$10,$V$11,$V$12,$V$13,$V$14,$V$15,$V$16,$V$17,$V$18)</f>
+        <v>0</v>
+      </c>
+      <c r="W19" s="11">
+        <f>SUM($W$3,$W$4,$W$5,$W$6,$W$7,$W$8,$W$9,$W$10,$W$11,$W$12,$W$13,$W$14,$W$15,$W$16,$W$17,$W$18)</f>
+        <v>0</v>
+      </c>
+      <c r="X19" s="11">
+        <f>SUM($X$3,$X$4,$X$5,$X$6,$X$7,$X$8,$X$9,$X$10,$X$11,$X$12,$X$13,$X$14,$X$15,$X$16,$X$17,$X$18)</f>
+        <v>0</v>
+      </c>
+      <c r="Y19" s="11">
+        <f>SUM($Y$3,$Y$4,$Y$5,$Y$6,$Y$7,$Y$8,$Y$9,$Y$10,$Y$11,$Y$12,$Y$13,$Y$14,$Y$15,$Y$16,$Y$17,$Y$18)</f>
+        <v>0</v>
+      </c>
+      <c r="Z19" s="6">
+        <f>SUM($Z$3,$Z$4,$Z$5,$Z$6,$Z$7,$Z$8,$Z$9,$Z$10,$Z$11,$Z$12,$Z$13,$Z$14,$Z$15,$Z$16,$Z$17,$Z$18)</f>
         <v>67000</v>
       </c>
-      <c r="T19" s="6">
-        <f>SUM($T$2,$T$3,$T$4,$T$5,$T$6,$T$7,$T$8,$T$9,$T$10,$T$11,$T$12,$T$13,$T$14,$T$15,$T$16,$T$17,$T$18)</f>
+      <c r="AA19" s="6">
+        <f>SUM($AA$3,$AA$4,$AA$5,$AA$6,$AA$7,$AA$8,$AA$9,$AA$10,$AA$11,$AA$12,$AA$13,$AA$14,$AA$15,$AA$16,$AA$17,$AA$18)</f>
         <v>67000</v>
       </c>
-      <c r="U19" s="11">
-        <f>SUM($U$2,$U$3,$U$4,$U$5,$U$6,$U$7,$U$8,$U$9,$U$10,$U$11,$U$12,$U$13,$U$14,$U$15,$U$16,$U$17,$U$18)</f>
+      <c r="AB19" s="11">
+        <f>SUM($AB$3,$AB$4,$AB$5,$AB$6,$AB$7,$AB$8,$AB$9,$AB$10,$AB$11,$AB$12,$AB$13,$AB$14,$AB$15,$AB$16,$AB$17,$AB$18)</f>
         <v>67</v>
       </c>
-      <c r="V19" s="11">
-        <f>SUM($V$2,$V$3,$V$4,$V$5,$V$6,$V$7,$V$8,$V$9,$V$10,$V$11,$V$12,$V$13,$V$14,$V$15,$V$16,$V$17,$V$18)</f>
-        <v>0</v>
-      </c>
-      <c r="W19" s="11">
-        <f>SUM($W$2,$W$3,$W$4,$W$5,$W$6,$W$7,$W$8,$W$9,$W$10,$W$11,$W$12,$W$13,$W$14,$W$15,$W$16,$W$17,$W$18)</f>
-        <v>0</v>
-      </c>
-      <c r="X19" s="11">
-        <f>SUM($X$2,$X$3,$X$4,$X$5,$X$6,$X$7,$X$8,$X$9,$X$10,$X$11,$X$12,$X$13,$X$14,$X$15,$X$16,$X$17,$X$18)</f>
-        <v>0</v>
-      </c>
-      <c r="Y19" s="11">
-        <f>SUM($Y$2,$Y$3,$Y$4,$Y$5,$Y$6,$Y$7,$Y$8,$Y$9,$Y$10,$Y$11,$Y$12,$Y$13,$Y$14,$Y$15,$Y$16,$Y$17,$Y$18)</f>
-        <v>0</v>
-      </c>
-      <c r="Z19" s="6">
-        <f>SUM($Z$2,$Z$3,$Z$4,$Z$5,$Z$6,$Z$7,$Z$8,$Z$9,$Z$10,$Z$11,$Z$12,$Z$13,$Z$14,$Z$15,$Z$16,$Z$17,$Z$18)</f>
+      <c r="AC19" s="11">
+        <f>SUM($AC$3,$AC$4,$AC$5,$AC$6,$AC$7,$AC$8,$AC$9,$AC$10,$AC$11,$AC$12,$AC$13,$AC$14,$AC$15,$AC$16,$AC$17,$AC$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AD19" s="11">
+        <f>SUM($AD$3,$AD$4,$AD$5,$AD$6,$AD$7,$AD$8,$AD$9,$AD$10,$AD$11,$AD$12,$AD$13,$AD$14,$AD$15,$AD$16,$AD$17,$AD$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AE19" s="11">
+        <f>SUM($AE$3,$AE$4,$AE$5,$AE$6,$AE$7,$AE$8,$AE$9,$AE$10,$AE$11,$AE$12,$AE$13,$AE$14,$AE$15,$AE$16,$AE$17,$AE$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AF19" s="6">
+        <f>SUM($AF$3,$AF$4,$AF$5,$AF$6,$AF$7,$AF$8,$AF$9,$AF$10,$AF$11,$AF$12,$AF$13,$AF$14,$AF$15,$AF$16,$AF$17,$AF$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AG19" s="6">
+        <f>SUM($AG$3,$AG$4,$AG$5,$AG$6,$AG$7,$AG$8,$AG$9,$AG$10,$AG$11,$AG$12,$AG$13,$AG$14,$AG$15,$AG$16,$AG$17,$AG$18)</f>
+        <v>66000</v>
+      </c>
+      <c r="AH19" s="6">
+        <f>SUM($AH$3,$AH$4,$AH$5,$AH$6,$AH$7,$AH$8,$AH$9,$AH$10,$AH$11,$AH$12,$AH$13,$AH$14,$AH$15,$AH$16,$AH$17,$AH$18)</f>
+        <v>66000</v>
+      </c>
+      <c r="AI19" s="11">
+        <f>SUM($AI$3,$AI$4,$AI$5,$AI$6,$AI$7,$AI$8,$AI$9,$AI$10,$AI$11,$AI$12,$AI$13,$AI$14,$AI$15,$AI$16,$AI$17,$AI$18)</f>
+        <v>66</v>
+      </c>
+      <c r="AJ19" s="11">
+        <f>SUM($AJ$3,$AJ$4,$AJ$5,$AJ$6,$AJ$7,$AJ$8,$AJ$9,$AJ$10,$AJ$11,$AJ$12,$AJ$13,$AJ$14,$AJ$15,$AJ$16,$AJ$17,$AJ$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AK19" s="11">
+        <f>SUM($AK$3,$AK$4,$AK$5,$AK$6,$AK$7,$AK$8,$AK$9,$AK$10,$AK$11,$AK$12,$AK$13,$AK$14,$AK$15,$AK$16,$AK$17,$AK$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AL19" s="11">
+        <f>SUM($AL$3,$AL$4,$AL$5,$AL$6,$AL$7,$AL$8,$AL$9,$AL$10,$AL$11,$AL$12,$AL$13,$AL$14,$AL$15,$AL$16,$AL$17,$AL$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AM19" s="6">
+        <f>SUM($AM$3,$AM$4,$AM$5,$AM$6,$AM$7,$AM$8,$AM$9,$AM$10,$AM$11,$AM$12,$AM$13,$AM$14,$AM$15,$AM$16,$AM$17,$AM$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AN19" s="6">
+        <f>SUM($AN$3,$AN$4,$AN$5,$AN$6,$AN$7,$AN$8,$AN$9,$AN$10,$AN$11,$AN$12,$AN$13,$AN$14,$AN$15,$AN$16,$AN$17,$AN$18)</f>
+        <v>69000</v>
+      </c>
+      <c r="AO19" s="6">
+        <f>SUM($AO$3,$AO$4,$AO$5,$AO$6,$AO$7,$AO$8,$AO$9,$AO$10,$AO$11,$AO$12,$AO$13,$AO$14,$AO$15,$AO$16,$AO$17,$AO$18)</f>
+        <v>69000</v>
+      </c>
+      <c r="AP19" s="11">
+        <f>SUM($AP$3,$AP$4,$AP$5,$AP$6,$AP$7,$AP$8,$AP$9,$AP$10,$AP$11,$AP$12,$AP$13,$AP$14,$AP$15,$AP$16,$AP$17,$AP$18)</f>
+        <v>69</v>
+      </c>
+      <c r="AQ19" s="11">
+        <f>SUM($AQ$3,$AQ$4,$AQ$5,$AQ$6,$AQ$7,$AQ$8,$AQ$9,$AQ$10,$AQ$11,$AQ$12,$AQ$13,$AQ$14,$AQ$15,$AQ$16,$AQ$17,$AQ$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AR19" s="11">
+        <f>SUM($AR$3,$AR$4,$AR$5,$AR$6,$AR$7,$AR$8,$AR$9,$AR$10,$AR$11,$AR$12,$AR$13,$AR$14,$AR$15,$AR$16,$AR$17,$AR$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AS19" s="11">
+        <f>SUM($AS$3,$AS$4,$AS$5,$AS$6,$AS$7,$AS$8,$AS$9,$AS$10,$AS$11,$AS$12,$AS$13,$AS$14,$AS$15,$AS$16,$AS$17,$AS$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AT19" s="6">
+        <f>SUM($AT$3,$AT$4,$AT$5,$AT$6,$AT$7,$AT$8,$AT$9,$AT$10,$AT$11,$AT$12,$AT$13,$AT$14,$AT$15,$AT$16,$AT$17,$AT$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AU19" s="6">
+        <f>SUM($AU$3,$AU$4,$AU$5,$AU$6,$AU$7,$AU$8,$AU$9,$AU$10,$AU$11,$AU$12,$AU$13,$AU$14,$AU$15,$AU$16,$AU$17,$AU$18)</f>
+        <v>69000</v>
+      </c>
+      <c r="AV19" s="6">
+        <f>SUM($AV$3,$AV$4,$AV$5,$AV$6,$AV$7,$AV$8,$AV$9,$AV$10,$AV$11,$AV$12,$AV$13,$AV$14,$AV$15,$AV$16,$AV$17,$AV$18)</f>
+        <v>69000</v>
+      </c>
+      <c r="AW19" s="11">
+        <f>SUM($AW$3,$AW$4,$AW$5,$AW$6,$AW$7,$AW$8,$AW$9,$AW$10,$AW$11,$AW$12,$AW$13,$AW$14,$AW$15,$AW$16,$AW$17,$AW$18)</f>
+        <v>69</v>
+      </c>
+      <c r="AX19" s="11">
+        <f>SUM($AX$3,$AX$4,$AX$5,$AX$6,$AX$7,$AX$8,$AX$9,$AX$10,$AX$11,$AX$12,$AX$13,$AX$14,$AX$15,$AX$16,$AX$17,$AX$18)</f>
+        <v>212.75</v>
+      </c>
+      <c r="AY19" s="11">
+        <f>SUM($AY$3,$AY$4,$AY$5,$AY$6,$AY$7,$AY$8,$AY$9,$AY$10,$AY$11,$AY$12,$AY$13,$AY$14,$AY$15,$AY$16,$AY$17,$AY$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AZ19" s="11">
+        <f>SUM($AZ$3,$AZ$4,$AZ$5,$AZ$6,$AZ$7,$AZ$8,$AZ$9,$AZ$10,$AZ$11,$AZ$12,$AZ$13,$AZ$14,$AZ$15,$AZ$16,$AZ$17,$AZ$18)</f>
+        <v>0</v>
+      </c>
+      <c r="BA19" s="6">
+        <f>SUM($BA$3,$BA$4,$BA$5,$BA$6,$BA$7,$BA$8,$BA$9,$BA$10,$BA$11,$BA$12,$BA$13,$BA$14,$BA$15,$BA$16,$BA$17,$BA$18)</f>
+        <v>0</v>
+      </c>
+      <c r="BB19" s="6">
+        <f>SUM($BB$3,$BB$4,$BB$5,$BB$6,$BB$7,$BB$8,$BB$9,$BB$10,$BB$11,$BB$12,$BB$13,$BB$14,$BB$15,$BB$16,$BB$17,$BB$18)</f>
         <v>72000</v>
       </c>
-      <c r="AA19" s="6">
-        <f>SUM($AA$2,$AA$3,$AA$4,$AA$5,$AA$6,$AA$7,$AA$8,$AA$9,$AA$10,$AA$11,$AA$12,$AA$13,$AA$14,$AA$15,$AA$16,$AA$17,$AA$18)</f>
+      <c r="BC19" s="6">
+        <f>SUM($BC$3,$BC$4,$BC$5,$BC$6,$BC$7,$BC$8,$BC$9,$BC$10,$BC$11,$BC$12,$BC$13,$BC$14,$BC$15,$BC$16,$BC$17,$BC$18)</f>
         <v>72000</v>
       </c>
-      <c r="AB19" s="11">
-        <f>SUM($AB$2,$AB$3,$AB$4,$AB$5,$AB$6,$AB$7,$AB$8,$AB$9,$AB$10,$AB$11,$AB$12,$AB$13,$AB$14,$AB$15,$AB$16,$AB$17,$AB$18)</f>
+      <c r="BD19" s="11">
+        <f>SUM($BD$3,$BD$4,$BD$5,$BD$6,$BD$7,$BD$8,$BD$9,$BD$10,$BD$11,$BD$12,$BD$13,$BD$14,$BD$15,$BD$16,$BD$17,$BD$18)</f>
         <v>72</v>
       </c>
-      <c r="AC19" s="11">
-        <f>SUM($AC$2,$AC$3,$AC$4,$AC$5,$AC$6,$AC$7,$AC$8,$AC$9,$AC$10,$AC$11,$AC$12,$AC$13,$AC$14,$AC$15,$AC$16,$AC$17,$AC$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AD19" s="11">
-        <f>SUM($AD$2,$AD$3,$AD$4,$AD$5,$AD$6,$AD$7,$AD$8,$AD$9,$AD$10,$AD$11,$AD$12,$AD$13,$AD$14,$AD$15,$AD$16,$AD$17,$AD$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AE19" s="11">
-        <f>SUM($AE$2,$AE$3,$AE$4,$AE$5,$AE$6,$AE$7,$AE$8,$AE$9,$AE$10,$AE$11,$AE$12,$AE$13,$AE$14,$AE$15,$AE$16,$AE$17,$AE$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AF19" s="6">
-        <f>SUM($AF$2,$AF$3,$AF$4,$AF$5,$AF$6,$AF$7,$AF$8,$AF$9,$AF$10,$AF$11,$AF$12,$AF$13,$AF$14,$AF$15,$AF$16,$AF$17,$AF$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AG19" s="6">
-        <f>SUM($AG$2,$AG$3,$AG$4,$AG$5,$AG$6,$AG$7,$AG$8,$AG$9,$AG$10,$AG$11,$AG$12,$AG$13,$AG$14,$AG$15,$AG$16,$AG$17,$AG$18)</f>
-        <v>69000</v>
-      </c>
-      <c r="AH19" s="6">
-        <f>SUM($AH$2,$AH$3,$AH$4,$AH$5,$AH$6,$AH$7,$AH$8,$AH$9,$AH$10,$AH$11,$AH$12,$AH$13,$AH$14,$AH$15,$AH$16,$AH$17,$AH$18)</f>
-        <v>69000</v>
-      </c>
-      <c r="AI19" s="11">
-        <f>SUM($AI$2,$AI$3,$AI$4,$AI$5,$AI$6,$AI$7,$AI$8,$AI$9,$AI$10,$AI$11,$AI$12,$AI$13,$AI$14,$AI$15,$AI$16,$AI$17,$AI$18)</f>
-        <v>69</v>
-      </c>
-      <c r="AJ19" s="11">
-        <f>SUM($AJ$2,$AJ$3,$AJ$4,$AJ$5,$AJ$6,$AJ$7,$AJ$8,$AJ$9,$AJ$10,$AJ$11,$AJ$12,$AJ$13,$AJ$14,$AJ$15,$AJ$16,$AJ$17,$AJ$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AK19" s="11">
-        <f>SUM($AK$2,$AK$3,$AK$4,$AK$5,$AK$6,$AK$7,$AK$8,$AK$9,$AK$10,$AK$11,$AK$12,$AK$13,$AK$14,$AK$15,$AK$16,$AK$17,$AK$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AL19" s="11">
-        <f>SUM($AL$2,$AL$3,$AL$4,$AL$5,$AL$6,$AL$7,$AL$8,$AL$9,$AL$10,$AL$11,$AL$12,$AL$13,$AL$14,$AL$15,$AL$16,$AL$17,$AL$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AM19" s="6">
-        <f>SUM($AM$2,$AM$3,$AM$4,$AM$5,$AM$6,$AM$7,$AM$8,$AM$9,$AM$10,$AM$11,$AM$12,$AM$13,$AM$14,$AM$15,$AM$16,$AM$17,$AM$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AN19" s="6">
-        <f>SUM($AN$2,$AN$3,$AN$4,$AN$5,$AN$6,$AN$7,$AN$8,$AN$9,$AN$10,$AN$11,$AN$12,$AN$13,$AN$14,$AN$15,$AN$16,$AN$17,$AN$18)</f>
+      <c r="BE19" s="11">
+        <f>SUM($BE$3,$BE$4,$BE$5,$BE$6,$BE$7,$BE$8,$BE$9,$BE$10,$BE$11,$BE$12,$BE$13,$BE$14,$BE$15,$BE$16,$BE$17,$BE$18)</f>
+        <v>0</v>
+      </c>
+      <c r="BF19" s="11">
+        <f>SUM($BF$3,$BF$4,$BF$5,$BF$6,$BF$7,$BF$8,$BF$9,$BF$10,$BF$11,$BF$12,$BF$13,$BF$14,$BF$15,$BF$16,$BF$17,$BF$18)</f>
+        <v>0</v>
+      </c>
+      <c r="BG19" s="11">
+        <f>SUM($BG$3,$BG$4,$BG$5,$BG$6,$BG$7,$BG$8,$BG$9,$BG$10,$BG$11,$BG$12,$BG$13,$BG$14,$BG$15,$BG$16,$BG$17,$BG$18)</f>
+        <v>0</v>
+      </c>
+      <c r="BH19" s="6">
+        <f>SUM($BH$3,$BH$4,$BH$5,$BH$6,$BH$7,$BH$8,$BH$9,$BH$10,$BH$11,$BH$12,$BH$13,$BH$14,$BH$15,$BH$16,$BH$17,$BH$18)</f>
+        <v>0</v>
+      </c>
+      <c r="BI19" s="6">
+        <f>SUM($BI$3,$BI$4,$BI$5,$BI$6,$BI$7,$BI$8,$BI$9,$BI$10,$BI$11,$BI$12,$BI$13,$BI$14,$BI$15,$BI$16,$BI$17,$BI$18)</f>
         <v>72000</v>
       </c>
-      <c r="AO19" s="6">
-        <f>SUM($AO$2,$AO$3,$AO$4,$AO$5,$AO$6,$AO$7,$AO$8,$AO$9,$AO$10,$AO$11,$AO$12,$AO$13,$AO$14,$AO$15,$AO$16,$AO$17,$AO$18)</f>
+      <c r="BJ19" s="6">
+        <f>SUM($BJ$3,$BJ$4,$BJ$5,$BJ$6,$BJ$7,$BJ$8,$BJ$9,$BJ$10,$BJ$11,$BJ$12,$BJ$13,$BJ$14,$BJ$15,$BJ$16,$BJ$17,$BJ$18)</f>
         <v>72000</v>
       </c>
-      <c r="AP19" s="11">
-        <f>SUM($AP$2,$AP$3,$AP$4,$AP$5,$AP$6,$AP$7,$AP$8,$AP$9,$AP$10,$AP$11,$AP$12,$AP$13,$AP$14,$AP$15,$AP$16,$AP$17,$AP$18)</f>
+      <c r="BK19" s="11">
+        <f>SUM($BK$3,$BK$4,$BK$5,$BK$6,$BK$7,$BK$8,$BK$9,$BK$10,$BK$11,$BK$12,$BK$13,$BK$14,$BK$15,$BK$16,$BK$17,$BK$18)</f>
         <v>72</v>
       </c>
-      <c r="AQ19" s="11">
-        <f>SUM($AQ$2,$AQ$3,$AQ$4,$AQ$5,$AQ$6,$AQ$7,$AQ$8,$AQ$9,$AQ$10,$AQ$11,$AQ$12,$AQ$13,$AQ$14,$AQ$15,$AQ$16,$AQ$17,$AQ$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AR19" s="11">
-        <f>SUM($AR$2,$AR$3,$AR$4,$AR$5,$AR$6,$AR$7,$AR$8,$AR$9,$AR$10,$AR$11,$AR$12,$AR$13,$AR$14,$AR$15,$AR$16,$AR$17,$AR$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AS19" s="11">
-        <f>SUM($AS$2,$AS$3,$AS$4,$AS$5,$AS$6,$AS$7,$AS$8,$AS$9,$AS$10,$AS$11,$AS$12,$AS$13,$AS$14,$AS$15,$AS$16,$AS$17,$AS$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AT19" s="6">
-        <f>SUM($AT$2,$AT$3,$AT$4,$AT$5,$AT$6,$AT$7,$AT$8,$AT$9,$AT$10,$AT$11,$AT$12,$AT$13,$AT$14,$AT$15,$AT$16,$AT$17,$AT$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AU19" s="6">
-        <f>SUM($AU$2,$AU$3,$AU$4,$AU$5,$AU$6,$AU$7,$AU$8,$AU$9,$AU$10,$AU$11,$AU$12,$AU$13,$AU$14,$AU$15,$AU$16,$AU$17,$AU$18)</f>
-        <v>72000</v>
-      </c>
-      <c r="AV19" s="6">
-        <f>SUM($AV$2,$AV$3,$AV$4,$AV$5,$AV$6,$AV$7,$AV$8,$AV$9,$AV$10,$AV$11,$AV$12,$AV$13,$AV$14,$AV$15,$AV$16,$AV$17,$AV$18)</f>
-        <v>72000</v>
-      </c>
-      <c r="AW19" s="11">
-        <f>SUM($AW$2,$AW$3,$AW$4,$AW$5,$AW$6,$AW$7,$AW$8,$AW$9,$AW$10,$AW$11,$AW$12,$AW$13,$AW$14,$AW$15,$AW$16,$AW$17,$AW$18)</f>
-        <v>72</v>
-      </c>
-      <c r="AX19" s="11">
-        <f>SUM($AX$2,$AX$3,$AX$4,$AX$5,$AX$6,$AX$7,$AX$8,$AX$9,$AX$10,$AX$11,$AX$12,$AX$13,$AX$14,$AX$15,$AX$16,$AX$17,$AX$18)</f>
-        <v>818.01</v>
-      </c>
-      <c r="AY19" s="11">
-        <f>SUM($AY$2,$AY$3,$AY$4,$AY$5,$AY$6,$AY$7,$AY$8,$AY$9,$AY$10,$AY$11,$AY$12,$AY$13,$AY$14,$AY$15,$AY$16,$AY$17,$AY$18)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ19" s="11">
-        <f>SUM($AZ$2,$AZ$3,$AZ$4,$AZ$5,$AZ$6,$AZ$7,$AZ$8,$AZ$9,$AZ$10,$AZ$11,$AZ$12,$AZ$13,$AZ$14,$AZ$15,$AZ$16,$AZ$17,$AZ$18)</f>
-        <v>0</v>
-      </c>
-      <c r="BA19" s="6">
-        <f>SUM($BA$2,$BA$3,$BA$4,$BA$5,$BA$6,$BA$7,$BA$8,$BA$9,$BA$10,$BA$11,$BA$12,$BA$13,$BA$14,$BA$15,$BA$16,$BA$17,$BA$18)</f>
-        <v>0</v>
-      </c>
-      <c r="BB19" s="6">
-        <f>SUM($BB$2,$BB$3,$BB$4,$BB$5,$BB$6,$BB$7,$BB$8,$BB$9,$BB$10,$BB$11,$BB$12,$BB$13,$BB$14,$BB$15,$BB$16,$BB$17,$BB$18)</f>
-        <v>76000</v>
-      </c>
-      <c r="BC19" s="6">
-        <f>SUM($BC$2,$BC$3,$BC$4,$BC$5,$BC$6,$BC$7,$BC$8,$BC$9,$BC$10,$BC$11,$BC$12,$BC$13,$BC$14,$BC$15,$BC$16,$BC$17,$BC$18)</f>
-        <v>76000</v>
-      </c>
-      <c r="BD19" s="11">
-        <f>SUM($BD$2,$BD$3,$BD$4,$BD$5,$BD$6,$BD$7,$BD$8,$BD$9,$BD$10,$BD$11,$BD$12,$BD$13,$BD$14,$BD$15,$BD$16,$BD$17,$BD$18)</f>
-        <v>76</v>
-      </c>
-      <c r="BE19" s="11">
-        <f>SUM($BE$2,$BE$3,$BE$4,$BE$5,$BE$6,$BE$7,$BE$8,$BE$9,$BE$10,$BE$11,$BE$12,$BE$13,$BE$14,$BE$15,$BE$16,$BE$17,$BE$18)</f>
-        <v>0</v>
-      </c>
-      <c r="BF19" s="11">
-        <f>SUM($BF$2,$BF$3,$BF$4,$BF$5,$BF$6,$BF$7,$BF$8,$BF$9,$BF$10,$BF$11,$BF$12,$BF$13,$BF$14,$BF$15,$BF$16,$BF$17,$BF$18)</f>
-        <v>0</v>
-      </c>
-      <c r="BG19" s="11">
-        <f>SUM($BG$2,$BG$3,$BG$4,$BG$5,$BG$6,$BG$7,$BG$8,$BG$9,$BG$10,$BG$11,$BG$12,$BG$13,$BG$14,$BG$15,$BG$16,$BG$17,$BG$18)</f>
-        <v>0</v>
-      </c>
-      <c r="BH19" s="6">
-        <f>SUM($BH$2,$BH$3,$BH$4,$BH$5,$BH$6,$BH$7,$BH$8,$BH$9,$BH$10,$BH$11,$BH$12,$BH$13,$BH$14,$BH$15,$BH$16,$BH$17,$BH$18)</f>
-        <v>0</v>
-      </c>
-      <c r="BI19" s="6">
-        <f>SUM($BI$2,$BI$3,$BI$4,$BI$5,$BI$6,$BI$7,$BI$8,$BI$9,$BI$10,$BI$11,$BI$12,$BI$13,$BI$14,$BI$15,$BI$16,$BI$17,$BI$18)</f>
-        <v>76000</v>
-      </c>
-      <c r="BJ19" s="6">
-        <f>SUM($BJ$2,$BJ$3,$BJ$4,$BJ$5,$BJ$6,$BJ$7,$BJ$8,$BJ$9,$BJ$10,$BJ$11,$BJ$12,$BJ$13,$BJ$14,$BJ$15,$BJ$16,$BJ$17,$BJ$18)</f>
-        <v>76000</v>
-      </c>
-      <c r="BK19" s="11">
-        <f>SUM($BK$2,$BK$3,$BK$4,$BK$5,$BK$6,$BK$7,$BK$8,$BK$9,$BK$10,$BK$11,$BK$12,$BK$13,$BK$14,$BK$15,$BK$16,$BK$17,$BK$18)</f>
-        <v>76</v>
-      </c>
       <c r="BL19" s="11">
-        <f>SUM($BL$2,$BL$3,$BL$4,$BL$5,$BL$6,$BL$7,$BL$8,$BL$9,$BL$10,$BL$11,$BL$12,$BL$13,$BL$14,$BL$15,$BL$16,$BL$17,$BL$18)</f>
+        <f>SUM($BL$3,$BL$4,$BL$5,$BL$6,$BL$7,$BL$8,$BL$9,$BL$10,$BL$11,$BL$12,$BL$13,$BL$14,$BL$15,$BL$16,$BL$17,$BL$18)</f>
         <v>0</v>
       </c>
       <c r="BM19" s="11">
-        <f>SUM($BM$2,$BM$3,$BM$4,$BM$5,$BM$6,$BM$7,$BM$8,$BM$9,$BM$10,$BM$11,$BM$12,$BM$13,$BM$14,$BM$15,$BM$16,$BM$17,$BM$18)</f>
+        <f>SUM($BM$3,$BM$4,$BM$5,$BM$6,$BM$7,$BM$8,$BM$9,$BM$10,$BM$11,$BM$12,$BM$13,$BM$14,$BM$15,$BM$16,$BM$17,$BM$18)</f>
         <v>0</v>
       </c>
       <c r="BN19" s="6">
-        <f>SUM($BN$2,$BN$3,$BN$4,$BN$5,$BN$6,$BN$7,$BN$8,$BN$9,$BN$10,$BN$11,$BN$12,$BN$13,$BN$14,$BN$15,$BN$16,$BN$17,$BN$18)</f>
-        <v>68000</v>
+        <f>SUM($BN$3,$BN$4,$BN$5,$BN$6,$BN$7,$BN$8,$BN$9,$BN$10,$BN$11,$BN$12,$BN$13,$BN$14,$BN$15,$BN$16,$BN$17,$BN$18)</f>
+        <v>66000</v>
       </c>
       <c r="BO19" s="6">
-        <f>SUM($BO$2,$BO$3,$BO$4,$BO$5,$BO$6,$BO$7,$BO$8,$BO$9,$BO$10,$BO$11,$BO$12,$BO$13,$BO$14,$BO$15,$BO$16,$BO$17,$BO$18)</f>
-        <v>68000</v>
+        <f>SUM($BO$3,$BO$4,$BO$5,$BO$6,$BO$7,$BO$8,$BO$9,$BO$10,$BO$11,$BO$12,$BO$13,$BO$14,$BO$15,$BO$16,$BO$17,$BO$18)</f>
+        <v>66000</v>
       </c>
       <c r="BP19" s="11">
-        <f>SUM($BP$2,$BP$3,$BP$4,$BP$5,$BP$6,$BP$7,$BP$8,$BP$9,$BP$10,$BP$11,$BP$12,$BP$13,$BP$14,$BP$15,$BP$16,$BP$17,$BP$18)</f>
-        <v>68</v>
+        <f>SUM($BP$3,$BP$4,$BP$5,$BP$6,$BP$7,$BP$8,$BP$9,$BP$10,$BP$11,$BP$12,$BP$13,$BP$14,$BP$15,$BP$16,$BP$17,$BP$18)</f>
+        <v>66</v>
       </c>
       <c r="BQ19" s="11">
-        <f>SUM($BQ$2,$BQ$3,$BQ$4,$BQ$5,$BQ$6,$BQ$7,$BQ$8,$BQ$9,$BQ$10,$BQ$11,$BQ$12,$BQ$13,$BQ$14,$BQ$15,$BQ$16,$BQ$17,$BQ$18)</f>
+        <f>SUM($BQ$3,$BQ$4,$BQ$5,$BQ$6,$BQ$7,$BQ$8,$BQ$9,$BQ$10,$BQ$11,$BQ$12,$BQ$13,$BQ$14,$BQ$15,$BQ$16,$BQ$17,$BQ$18)</f>
         <v>0</v>
       </c>
       <c r="BR19" s="11">
-        <f>SUM($BR$2,$BR$3,$BR$4,$BR$5,$BR$6,$BR$7,$BR$8,$BR$9,$BR$10,$BR$11,$BR$12,$BR$13,$BR$14,$BR$15,$BR$16,$BR$17,$BR$18)</f>
+        <f>SUM($BR$3,$BR$4,$BR$5,$BR$6,$BR$7,$BR$8,$BR$9,$BR$10,$BR$11,$BR$12,$BR$13,$BR$14,$BR$15,$BR$16,$BR$17,$BR$18)</f>
         <v>0</v>
       </c>
       <c r="BS19" s="6">
-        <f>SUM($BS$2,$BS$3,$BS$4,$BS$5,$BS$6,$BS$7,$BS$8,$BS$9,$BS$10,$BS$11,$BS$12,$BS$13,$BS$14,$BS$15,$BS$16,$BS$17,$BS$18)</f>
-        <v>78000</v>
+        <f>SUM($BS$3,$BS$4,$BS$5,$BS$6,$BS$7,$BS$8,$BS$9,$BS$10,$BS$11,$BS$12,$BS$13,$BS$14,$BS$15,$BS$16,$BS$17,$BS$18)</f>
+        <v>74000</v>
       </c>
       <c r="BT19" s="6">
-        <f>SUM($BT$2,$BT$3,$BT$4,$BT$5,$BT$6,$BT$7,$BT$8,$BT$9,$BT$10,$BT$11,$BT$12,$BT$13,$BT$14,$BT$15,$BT$16,$BT$17,$BT$18)</f>
-        <v>78000</v>
+        <f>SUM($BT$3,$BT$4,$BT$5,$BT$6,$BT$7,$BT$8,$BT$9,$BT$10,$BT$11,$BT$12,$BT$13,$BT$14,$BT$15,$BT$16,$BT$17,$BT$18)</f>
+        <v>74000</v>
       </c>
       <c r="BU19" s="11">
-        <f>SUM($BU$2,$BU$3,$BU$4,$BU$5,$BU$6,$BU$7,$BU$8,$BU$9,$BU$10,$BU$11,$BU$12,$BU$13,$BU$14,$BU$15,$BU$16,$BU$17,$BU$18)</f>
-        <v>78</v>
+        <f>SUM($BU$3,$BU$4,$BU$5,$BU$6,$BU$7,$BU$8,$BU$9,$BU$10,$BU$11,$BU$12,$BU$13,$BU$14,$BU$15,$BU$16,$BU$17,$BU$18)</f>
+        <v>74</v>
       </c>
       <c r="BV19" s="11">
-        <f>SUM($BV$2,$BV$3,$BV$4,$BV$5,$BV$6,$BV$7,$BV$8,$BV$9,$BV$10,$BV$11,$BV$12,$BV$13,$BV$14,$BV$15,$BV$16,$BV$17,$BV$18)</f>
+        <f>SUM($BV$3,$BV$4,$BV$5,$BV$6,$BV$7,$BV$8,$BV$9,$BV$10,$BV$11,$BV$12,$BV$13,$BV$14,$BV$15,$BV$16,$BV$17,$BV$18)</f>
         <v>0</v>
       </c>
       <c r="BW19" s="11">
-        <f>SUM($BW$2,$BW$3,$BW$4,$BW$5,$BW$6,$BW$7,$BW$8,$BW$9,$BW$10,$BW$11,$BW$12,$BW$13,$BW$14,$BW$15,$BW$16,$BW$17,$BW$18)</f>
+        <f>SUM($BW$3,$BW$4,$BW$5,$BW$6,$BW$7,$BW$8,$BW$9,$BW$10,$BW$11,$BW$12,$BW$13,$BW$14,$BW$15,$BW$16,$BW$17,$BW$18)</f>
         <v>0</v>
       </c>
       <c r="BX19" s="6">
-        <f>SUM($BX$2,$BX$3,$BX$4,$BX$5,$BX$6,$BX$7,$BX$8,$BX$9,$BX$10,$BX$11,$BX$12,$BX$13,$BX$14,$BX$15,$BX$16,$BX$17,$BX$18)</f>
-        <v>78000</v>
+        <f>SUM($BX$3,$BX$4,$BX$5,$BX$6,$BX$7,$BX$8,$BX$9,$BX$10,$BX$11,$BX$12,$BX$13,$BX$14,$BX$15,$BX$16,$BX$17,$BX$18)</f>
+        <v>74000</v>
       </c>
       <c r="BY19" s="6">
-        <f>SUM($BY$2,$BY$3,$BY$4,$BY$5,$BY$6,$BY$7,$BY$8,$BY$9,$BY$10,$BY$11,$BY$12,$BY$13,$BY$14,$BY$15,$BY$16,$BY$17,$BY$18)</f>
-        <v>78000</v>
+        <f>SUM($BY$3,$BY$4,$BY$5,$BY$6,$BY$7,$BY$8,$BY$9,$BY$10,$BY$11,$BY$12,$BY$13,$BY$14,$BY$15,$BY$16,$BY$17,$BY$18)</f>
+        <v>74000</v>
       </c>
       <c r="BZ19" s="11">
-        <f>SUM($BZ$2,$BZ$3,$BZ$4,$BZ$5,$BZ$6,$BZ$7,$BZ$8,$BZ$9,$BZ$10,$BZ$11,$BZ$12,$BZ$13,$BZ$14,$BZ$15,$BZ$16,$BZ$17,$BZ$18)</f>
-        <v>78</v>
+        <f>SUM($BZ$3,$BZ$4,$BZ$5,$BZ$6,$BZ$7,$BZ$8,$BZ$9,$BZ$10,$BZ$11,$BZ$12,$BZ$13,$BZ$14,$BZ$15,$BZ$16,$BZ$17,$BZ$18)</f>
+        <v>74</v>
       </c>
       <c r="CA19" s="11">
-        <f>SUM($CA$2,$CA$3,$CA$4,$CA$5,$CA$6,$CA$7,$CA$8,$CA$9,$CA$10,$CA$11,$CA$12,$CA$13,$CA$14,$CA$15,$CA$16,$CA$17,$CA$18)</f>
+        <f>SUM($CA$3,$CA$4,$CA$5,$CA$6,$CA$7,$CA$8,$CA$9,$CA$10,$CA$11,$CA$12,$CA$13,$CA$14,$CA$15,$CA$16,$CA$17,$CA$18)</f>
         <v>0</v>
       </c>
       <c r="CB19" s="11">
-        <f>SUM($CB$2,$CB$3,$CB$4,$CB$5,$CB$6,$CB$7,$CB$8,$CB$9,$CB$10,$CB$11,$CB$12,$CB$13,$CB$14,$CB$15,$CB$16,$CB$17,$CB$18)</f>
+        <f>SUM($CB$3,$CB$4,$CB$5,$CB$6,$CB$7,$CB$8,$CB$9,$CB$10,$CB$11,$CB$12,$CB$13,$CB$14,$CB$15,$CB$16,$CB$17,$CB$18)</f>
         <v>0</v>
       </c>
       <c r="CC19" s="6">
-        <f>SUM($CC$2,$CC$3,$CC$4,$CC$5,$CC$6,$CC$7,$CC$8,$CC$9,$CC$10,$CC$11,$CC$12,$CC$13,$CC$14,$CC$15,$CC$16,$CC$17,$CC$18)</f>
-        <v>78000</v>
+        <f>SUM($CC$3,$CC$4,$CC$5,$CC$6,$CC$7,$CC$8,$CC$9,$CC$10,$CC$11,$CC$12,$CC$13,$CC$14,$CC$15,$CC$16,$CC$17,$CC$18)</f>
+        <v>74000</v>
       </c>
       <c r="CD19" s="6">
-        <f>SUM($CD$2,$CD$3,$CD$4,$CD$5,$CD$6,$CD$7,$CD$8,$CD$9,$CD$10,$CD$11,$CD$12,$CD$13,$CD$14,$CD$15,$CD$16,$CD$17,$CD$18)</f>
-        <v>78000</v>
+        <f>SUM($CD$3,$CD$4,$CD$5,$CD$6,$CD$7,$CD$8,$CD$9,$CD$10,$CD$11,$CD$12,$CD$13,$CD$14,$CD$15,$CD$16,$CD$17,$CD$18)</f>
+        <v>74000</v>
       </c>
       <c r="CE19" s="11">
-        <f>SUM($CE$2,$CE$3,$CE$4,$CE$5,$CE$6,$CE$7,$CE$8,$CE$9,$CE$10,$CE$11,$CE$12,$CE$13,$CE$14,$CE$15,$CE$16,$CE$17,$CE$18)</f>
-        <v>78</v>
+        <f>SUM($CE$3,$CE$4,$CE$5,$CE$6,$CE$7,$CE$8,$CE$9,$CE$10,$CE$11,$CE$12,$CE$13,$CE$14,$CE$15,$CE$16,$CE$17,$CE$18)</f>
+        <v>74</v>
       </c>
       <c r="CF19" s="11">
-        <f>SUM($CF$2,$CF$3,$CF$4,$CF$5,$CF$6,$CF$7,$CF$8,$CF$9,$CF$10,$CF$11,$CF$12,$CF$13,$CF$14,$CF$15,$CF$16,$CF$17,$CF$18)</f>
+        <f>SUM($CF$3,$CF$4,$CF$5,$CF$6,$CF$7,$CF$8,$CF$9,$CF$10,$CF$11,$CF$12,$CF$13,$CF$14,$CF$15,$CF$16,$CF$17,$CF$18)</f>
         <v>0</v>
       </c>
       <c r="CG19" s="11">
-        <f>SUM($CG$2,$CG$3,$CG$4,$CG$5,$CG$6,$CG$7,$CG$8,$CG$9,$CG$10,$CG$11,$CG$12,$CG$13,$CG$14,$CG$15,$CG$16,$CG$17,$CG$18)</f>
+        <f>SUM($CG$3,$CG$4,$CG$5,$CG$6,$CG$7,$CG$8,$CG$9,$CG$10,$CG$11,$CG$12,$CG$13,$CG$14,$CG$15,$CG$16,$CG$17,$CG$18)</f>
         <v>0</v>
       </c>
       <c r="CH19" s="6">
-        <f>SUM($CH$2,$CH$3,$CH$4,$CH$5,$CH$6,$CH$7,$CH$8,$CH$9,$CH$10,$CH$11,$CH$12,$CH$13,$CH$14,$CH$15,$CH$16,$CH$17,$CH$18)</f>
-        <v>78000</v>
+        <f>SUM($CH$3,$CH$4,$CH$5,$CH$6,$CH$7,$CH$8,$CH$9,$CH$10,$CH$11,$CH$12,$CH$13,$CH$14,$CH$15,$CH$16,$CH$17,$CH$18)</f>
+        <v>74000</v>
       </c>
       <c r="CI19" s="6">
-        <f>SUM($CI$2,$CI$3,$CI$4,$CI$5,$CI$6,$CI$7,$CI$8,$CI$9,$CI$10,$CI$11,$CI$12,$CI$13,$CI$14,$CI$15,$CI$16,$CI$17,$CI$18)</f>
-        <v>78000</v>
+        <f>SUM($CI$3,$CI$4,$CI$5,$CI$6,$CI$7,$CI$8,$CI$9,$CI$10,$CI$11,$CI$12,$CI$13,$CI$14,$CI$15,$CI$16,$CI$17,$CI$18)</f>
+        <v>74000</v>
       </c>
       <c r="CJ19" s="11">
-        <f>SUM($CJ$2,$CJ$3,$CJ$4,$CJ$5,$CJ$6,$CJ$7,$CJ$8,$CJ$9,$CJ$10,$CJ$11,$CJ$12,$CJ$13,$CJ$14,$CJ$15,$CJ$16,$CJ$17,$CJ$18)</f>
-        <v>78</v>
+        <f>SUM($CJ$3,$CJ$4,$CJ$5,$CJ$6,$CJ$7,$CJ$8,$CJ$9,$CJ$10,$CJ$11,$CJ$12,$CJ$13,$CJ$14,$CJ$15,$CJ$16,$CJ$17,$CJ$18)</f>
+        <v>74</v>
       </c>
       <c r="CK19" s="11">
-        <f>SUM($CK$2,$CK$3,$CK$4,$CK$5,$CK$6,$CK$7,$CK$8,$CK$9,$CK$10,$CK$11,$CK$12,$CK$13,$CK$14,$CK$15,$CK$16,$CK$17,$CK$18)</f>
+        <f>SUM($CK$3,$CK$4,$CK$5,$CK$6,$CK$7,$CK$8,$CK$9,$CK$10,$CK$11,$CK$12,$CK$13,$CK$14,$CK$15,$CK$16,$CK$17,$CK$18)</f>
         <v>0</v>
       </c>
       <c r="CL19" s="11">
-        <f>SUM($CL$2,$CL$3,$CL$4,$CL$5,$CL$6,$CL$7,$CL$8,$CL$9,$CL$10,$CL$11,$CL$12,$CL$13,$CL$14,$CL$15,$CL$16,$CL$17,$CL$18)</f>
+        <f>SUM($CL$3,$CL$4,$CL$5,$CL$6,$CL$7,$CL$8,$CL$9,$CL$10,$CL$11,$CL$12,$CL$13,$CL$14,$CL$15,$CL$16,$CL$17,$CL$18)</f>
         <v>0</v>
       </c>
       <c r="CM19" s="11">
-        <f>SUM($CM$2,$CM$3,$CM$4,$CM$5,$CM$6,$CM$7,$CM$8,$CM$9,$CM$10,$CM$11,$CM$12,$CM$13,$CM$14,$CM$15,$CM$16,$CM$17,$CM$18)</f>
+        <f>SUM($CM$3,$CM$4,$CM$5,$CM$6,$CM$7,$CM$8,$CM$9,$CM$10,$CM$11,$CM$12,$CM$13,$CM$14,$CM$15,$CM$16,$CM$17,$CM$18)</f>
         <v>0</v>
       </c>
       <c r="CN19" s="7">
-        <f>SUM($CN$2,$CN$3,$CN$4,$CN$5,$CN$6,$CN$7,$CN$8,$CN$9,$CN$10,$CN$11,$CN$12,$CN$13,$CN$14,$CN$15,$CN$16,$CN$17,$CN$18)</f>
-        <v>884000</v>
+        <f>SUM($CN$3,$CN$4,$CN$5,$CN$6,$CN$7,$CN$8,$CN$9,$CN$10,$CN$11,$CN$12,$CN$13,$CN$14,$CN$15,$CN$16,$CN$17,$CN$18)</f>
+        <v>841000</v>
       </c>
       <c r="CO19" s="7">
-        <f>SUM($CO$2,$CO$3,$CO$4,$CO$5,$CO$6,$CO$7,$CO$8,$CO$9,$CO$10,$CO$11,$CO$12,$CO$13,$CO$14,$CO$15,$CO$16,$CO$17,$CO$18)</f>
-        <v>884000</v>
+        <f>SUM($CO$3,$CO$4,$CO$5,$CO$6,$CO$7,$CO$8,$CO$9,$CO$10,$CO$11,$CO$12,$CO$13,$CO$14,$CO$15,$CO$16,$CO$17,$CO$18)</f>
+        <v>841000</v>
       </c>
       <c r="CP19" s="11">
-        <f>SUM($CP$2,$CP$3,$CP$4,$CP$5,$CP$6,$CP$7,$CP$8,$CP$9,$CP$10,$CP$11,$CP$12,$CP$13,$CP$14,$CP$15,$CP$16,$CP$17,$CP$18)</f>
-        <v>72.999999999999986</v>
+        <f>SUM($CP$3,$CP$4,$CP$5,$CP$6,$CP$7,$CP$8,$CP$9,$CP$10,$CP$11,$CP$12,$CP$13,$CP$14,$CP$15,$CP$16,$CP$17,$CP$18)</f>
+        <v>69.499999999999986</v>
       </c>
       <c r="CQ19" s="11">
-        <f>SUM($CQ$2,$CQ$3,$CQ$4,$CQ$5,$CQ$6,$CQ$7,$CQ$8,$CQ$9,$CQ$10,$CQ$11,$CQ$12,$CQ$13,$CQ$14,$CQ$15,$CQ$16,$CQ$17,$CQ$18)</f>
+        <f>SUM($CQ$3,$CQ$4,$CQ$5,$CQ$6,$CQ$7,$CQ$8,$CQ$9,$CQ$10,$CQ$11,$CQ$12,$CQ$13,$CQ$14,$CQ$15,$CQ$16,$CQ$17,$CQ$18)</f>
         <v>0</v>
       </c>
       <c r="CR19" s="11">
-        <f>SUM($CR$2,$CR$3,$CR$4,$CR$5,$CR$6,$CR$7,$CR$8,$CR$9,$CR$10,$CR$11,$CR$12,$CR$13,$CR$14,$CR$15,$CR$16,$CR$17,$CR$18)</f>
+        <f>SUM($CR$3,$CR$4,$CR$5,$CR$6,$CR$7,$CR$8,$CR$9,$CR$10,$CR$11,$CR$12,$CR$13,$CR$14,$CR$15,$CR$16,$CR$17,$CR$18)</f>
         <v>0</v>
       </c>
       <c r="CS19" s="11">
-        <f>SUM($CS$2,$CS$3,$CS$4,$CS$5,$CS$6,$CS$7,$CS$8,$CS$9,$CS$10,$CS$11,$CS$12,$CS$13,$CS$14,$CS$15,$CS$16,$CS$17,$CS$18)</f>
+        <f>SUM($CS$3,$CS$4,$CS$5,$CS$6,$CS$7,$CS$8,$CS$9,$CS$10,$CS$11,$CS$12,$CS$13,$CS$14,$CS$15,$CS$16,$CS$17,$CS$18)</f>
         <v>0</v>
       </c>
       <c r="CT19" s="6">
-        <f>SUM($CT$2,$CT$3,$CT$4,$CT$5,$CT$6,$CT$7,$CT$8,$CT$9,$CT$10,$CT$11,$CT$12,$CT$13,$CT$14,$CT$15,$CT$16,$CT$17,$CT$18)</f>
-        <v>-884000</v>
+        <f>SUM($CT$3,$CT$4,$CT$5,$CT$6,$CT$7,$CT$8,$CT$9,$CT$10,$CT$11,$CT$12,$CT$13,$CT$14,$CT$15,$CT$16,$CT$17,$CT$18)</f>
+        <v>-841000</v>
       </c>
       <c r="CU19" s="6">
-        <f>SUM($CU$2,$CU$3,$CU$4,$CU$5,$CU$6,$CU$7,$CU$8,$CU$9,$CU$10,$CU$11,$CU$12,$CU$13,$CU$14,$CU$15,$CU$16,$CU$17,$CU$18)</f>
-        <v>-884000</v>
+        <f>SUM($CU$3,$CU$4,$CU$5,$CU$6,$CU$7,$CU$8,$CU$9,$CU$10,$CU$11,$CU$12,$CU$13,$CU$14,$CU$15,$CU$16,$CU$17,$CU$18)</f>
+        <v>-841000</v>
       </c>
       <c r="CV19" s="11">
-        <f>SUM($CV$2,$CV$3,$CV$4,$CV$5,$CV$6,$CV$7,$CV$8,$CV$9,$CV$10,$CV$11,$CV$12,$CV$13,$CV$14,$CV$15,$CV$16,$CV$17,$CV$18)</f>
+        <f>SUM($CV$3,$CV$4,$CV$5,$CV$6,$CV$7,$CV$8,$CV$9,$CV$10,$CV$11,$CV$12,$CV$13,$CV$14,$CV$15,$CV$16,$CV$17,$CV$18)</f>
         <v>0</v>
       </c>
       <c r="CW19" s="11">
-        <f>SUM($CW$2,$CW$3,$CW$4,$CW$5,$CW$6,$CW$7,$CW$8,$CW$9,$CW$10,$CW$11,$CW$12,$CW$13,$CW$14,$CW$15,$CW$16,$CW$17,$CW$18)</f>
+        <f>SUM($CW$3,$CW$4,$CW$5,$CW$6,$CW$7,$CW$8,$CW$9,$CW$10,$CW$11,$CW$12,$CW$13,$CW$14,$CW$15,$CW$16,$CW$17,$CW$18)</f>
         <v>0</v>
       </c>
       <c r="CX19" s="11">
-        <f>SUM($CX$2,$CX$3,$CX$4,$CX$5,$CX$6,$CX$7,$CX$8,$CX$9,$CX$10,$CX$11,$CX$12,$CX$13,$CX$14,$CX$15,$CX$16,$CX$17,$CX$18)</f>
+        <f>SUM($CX$3,$CX$4,$CX$5,$CX$6,$CX$7,$CX$8,$CX$9,$CX$10,$CX$11,$CX$12,$CX$13,$CX$14,$CX$15,$CX$16,$CX$17,$CX$18)</f>
         <v>0</v>
       </c>
       <c r="CY19" s="11">
-        <f>SUM($CY$2,$CY$3,$CY$4,$CY$5,$CY$6,$CY$7,$CY$8,$CY$9,$CY$10,$CY$11,$CY$12,$CY$13,$CY$14,$CY$15,$CY$16,$CY$17,$CY$18)</f>
+        <f>SUM($CY$3,$CY$4,$CY$5,$CY$6,$CY$7,$CY$8,$CY$9,$CY$10,$CY$11,$CY$12,$CY$13,$CY$14,$CY$15,$CY$16,$CY$17,$CY$18)</f>
         <v>0</v>
       </c>
       <c r="CZ19" s="6">
-        <f>SUM($CZ$2,$CZ$3,$CZ$4,$CZ$5,$CZ$6,$CZ$7,$CZ$8,$CZ$9,$CZ$10,$CZ$11,$CZ$12,$CZ$13,$CZ$14,$CZ$15,$CZ$16,$CZ$17,$CZ$18)</f>
-        <v>884000</v>
+        <f>SUM($CZ$3,$CZ$4,$CZ$5,$CZ$6,$CZ$7,$CZ$8,$CZ$9,$CZ$10,$CZ$11,$CZ$12,$CZ$13,$CZ$14,$CZ$15,$CZ$16,$CZ$17,$CZ$18)</f>
+        <v>841000</v>
       </c>
       <c r="DA19" s="6">
-        <f>SUM($DA$2,$DA$3,$DA$4,$DA$5,$DA$6,$DA$7,$DA$8,$DA$9,$DA$10,$DA$11,$DA$12,$DA$13,$DA$14,$DA$15,$DA$16,$DA$17,$DA$18)</f>
-        <v>884000</v>
+        <f>SUM($DA$3,$DA$4,$DA$5,$DA$6,$DA$7,$DA$8,$DA$9,$DA$10,$DA$11,$DA$12,$DA$13,$DA$14,$DA$15,$DA$16,$DA$17,$DA$18)</f>
+        <v>841000</v>
       </c>
     </row>
     <row r="20" spans="1:105" x14ac:dyDescent="0.3">
@@ -7417,20 +7422,20 @@
     </row>
     <row r="22" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>106</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>163</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>164</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G22" s="3">
         <v>5842263202</v>
@@ -7439,10 +7444,10 @@
         <v>109</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>157</v>
@@ -7726,7 +7731,7 @@
     </row>
     <row r="23" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>106</v>
@@ -7735,11 +7740,11 @@
         <v>107</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E23" s="8"/>
       <c r="F23" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G23" s="8">
         <v>5841813202</v>
@@ -7748,10 +7753,10 @@
         <v>109</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K23" s="8" t="s">
         <v>157</v>
@@ -8035,20 +8040,20 @@
     </row>
     <row r="24" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>106</v>
       </c>
       <c r="C24" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>163</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>164</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G24" s="3">
         <v>5842263202</v>
@@ -8057,10 +8062,10 @@
         <v>109</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K24" s="3" t="s">
         <v>157</v>
@@ -8344,7 +8349,7 @@
     </row>
     <row r="25" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>106</v>
@@ -8353,11 +8358,11 @@
         <v>107</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E25" s="8"/>
       <c r="F25" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G25" s="8">
         <v>5841813202</v>
@@ -8366,10 +8371,10 @@
         <v>109</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K25" s="8" t="s">
         <v>157</v>
@@ -8654,7 +8659,7 @@
     <row r="26" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
       <c r="B26" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
@@ -8668,8 +8673,14 @@
       <c r="L26" s="3"/>
       <c r="M26" s="4"/>
       <c r="N26" s="4"/>
-      <c r="O26" s="5"/>
-      <c r="P26" s="5"/>
+      <c r="O26" s="5">
+        <f>SUM($O$21:$O$25)</f>
+        <v>0</v>
+      </c>
+      <c r="P26" s="5">
+        <f>SUM($P$21:$P$25)</f>
+        <v>0</v>
+      </c>
       <c r="Q26" s="6">
         <f>SUM($Q$21:$Q$25)</f>
         <v>0</v>
@@ -9136,7 +9147,7 @@
     </row>
     <row r="28" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>106</v>
@@ -9449,7 +9460,7 @@
     </row>
     <row r="29" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="B29" s="8" t="s">
         <v>106</v>
@@ -9758,7 +9769,7 @@
     </row>
     <row r="30" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>106</v>
@@ -10067,7 +10078,7 @@
     </row>
     <row r="31" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="B31" s="8" t="s">
         <v>106</v>
@@ -10391,8 +10402,14 @@
       <c r="L32" s="3"/>
       <c r="M32" s="4"/>
       <c r="N32" s="4"/>
-      <c r="O32" s="5"/>
-      <c r="P32" s="5"/>
+      <c r="O32" s="5">
+        <f>SUM($O$28:$O$31)</f>
+        <v>0</v>
+      </c>
+      <c r="P32" s="5">
+        <f>SUM($P$28:$P$31)</f>
+        <v>0</v>
+      </c>
       <c r="Q32" s="6">
         <f>SUM($Q$28:$Q$31)</f>
         <v>0</v>
@@ -10750,96 +10767,112 @@
         <v>158000</v>
       </c>
     </row>
-    <row r="33" spans="17:105" x14ac:dyDescent="0.3">
-      <c r="Q33" s="12"/>
-      <c r="R33" s="12"/>
-      <c r="S33" s="12"/>
-      <c r="T33" s="12"/>
-      <c r="U33" s="12"/>
-      <c r="V33" s="12"/>
-      <c r="W33" s="12"/>
-      <c r="X33" s="12"/>
-      <c r="Y33" s="12"/>
-      <c r="Z33" s="12"/>
-      <c r="AA33" s="12"/>
-      <c r="AB33" s="12"/>
-      <c r="AC33" s="12"/>
-      <c r="AD33" s="12"/>
-      <c r="AE33" s="12"/>
-      <c r="AF33" s="12"/>
-      <c r="AG33" s="12"/>
-      <c r="AH33" s="12"/>
-      <c r="AI33" s="12"/>
-      <c r="AJ33" s="12"/>
-      <c r="AK33" s="12"/>
-      <c r="AL33" s="12"/>
-      <c r="AM33" s="12"/>
-      <c r="AN33" s="12"/>
-      <c r="AO33" s="12"/>
-      <c r="AP33" s="12"/>
-      <c r="AQ33" s="12"/>
-      <c r="AR33" s="12"/>
-      <c r="AS33" s="12"/>
-      <c r="AT33" s="12"/>
-      <c r="AU33" s="12"/>
-      <c r="AV33" s="12"/>
-      <c r="AW33" s="12"/>
-      <c r="AX33" s="12"/>
-      <c r="AY33" s="12"/>
-      <c r="AZ33" s="12"/>
-      <c r="BA33" s="12"/>
-      <c r="BB33" s="12"/>
-      <c r="BC33" s="12"/>
-      <c r="BD33" s="12"/>
-      <c r="BE33" s="12"/>
-      <c r="BF33" s="12"/>
-      <c r="BG33" s="12"/>
-      <c r="BH33" s="12"/>
-      <c r="BI33" s="12"/>
-      <c r="BJ33" s="12"/>
-      <c r="BK33" s="12"/>
-      <c r="BL33" s="12"/>
-      <c r="BM33" s="12"/>
-      <c r="BN33" s="12"/>
-      <c r="BO33" s="12"/>
-      <c r="BP33" s="12"/>
-      <c r="BQ33" s="12"/>
-      <c r="BR33" s="12"/>
-      <c r="BS33" s="12"/>
-      <c r="BT33" s="12"/>
-      <c r="BU33" s="12"/>
-      <c r="BV33" s="12"/>
-      <c r="BW33" s="12"/>
-      <c r="BX33" s="12"/>
-      <c r="BY33" s="12"/>
-      <c r="BZ33" s="12"/>
-      <c r="CA33" s="12"/>
-      <c r="CB33" s="12"/>
-      <c r="CC33" s="12"/>
-      <c r="CD33" s="12"/>
-      <c r="CE33" s="12"/>
-      <c r="CF33" s="12"/>
-      <c r="CG33" s="12"/>
-      <c r="CH33" s="12"/>
-      <c r="CI33" s="12"/>
-      <c r="CJ33" s="12"/>
-      <c r="CK33" s="12"/>
-      <c r="CL33" s="12"/>
-      <c r="CM33" s="12"/>
-      <c r="CN33" s="13"/>
-      <c r="CO33" s="13"/>
-      <c r="CP33" s="12"/>
-      <c r="CQ33" s="12"/>
-      <c r="CR33" s="12"/>
-      <c r="CS33" s="12"/>
-      <c r="CT33" s="12"/>
-      <c r="CU33" s="12"/>
-      <c r="CV33" s="12"/>
-      <c r="CW33" s="12"/>
-      <c r="CX33" s="12"/>
-      <c r="CY33" s="12"/>
-      <c r="CZ33" s="12"/>
-      <c r="DA33" s="12"/>
+    <row r="33" spans="1:105" x14ac:dyDescent="0.3">
+      <c r="A33" s="8"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="8"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="10"/>
+      <c r="P33" s="10"/>
+      <c r="Q33" s="11"/>
+      <c r="R33" s="11"/>
+      <c r="S33" s="6"/>
+      <c r="T33" s="6"/>
+      <c r="U33" s="11"/>
+      <c r="V33" s="11"/>
+      <c r="W33" s="11"/>
+      <c r="X33" s="11"/>
+      <c r="Y33" s="11"/>
+      <c r="Z33" s="6"/>
+      <c r="AA33" s="6"/>
+      <c r="AB33" s="11"/>
+      <c r="AC33" s="11"/>
+      <c r="AD33" s="11"/>
+      <c r="AE33" s="11"/>
+      <c r="AF33" s="6"/>
+      <c r="AG33" s="6"/>
+      <c r="AH33" s="6"/>
+      <c r="AI33" s="11"/>
+      <c r="AJ33" s="11"/>
+      <c r="AK33" s="11"/>
+      <c r="AL33" s="11"/>
+      <c r="AM33" s="6"/>
+      <c r="AN33" s="6"/>
+      <c r="AO33" s="6"/>
+      <c r="AP33" s="11"/>
+      <c r="AQ33" s="11"/>
+      <c r="AR33" s="11"/>
+      <c r="AS33" s="11"/>
+      <c r="AT33" s="6"/>
+      <c r="AU33" s="6"/>
+      <c r="AV33" s="6"/>
+      <c r="AW33" s="11"/>
+      <c r="AX33" s="11"/>
+      <c r="AY33" s="11"/>
+      <c r="AZ33" s="11"/>
+      <c r="BA33" s="6"/>
+      <c r="BB33" s="6"/>
+      <c r="BC33" s="6"/>
+      <c r="BD33" s="11"/>
+      <c r="BE33" s="11"/>
+      <c r="BF33" s="11"/>
+      <c r="BG33" s="11"/>
+      <c r="BH33" s="6"/>
+      <c r="BI33" s="6"/>
+      <c r="BJ33" s="6"/>
+      <c r="BK33" s="11"/>
+      <c r="BL33" s="11"/>
+      <c r="BM33" s="11"/>
+      <c r="BN33" s="6"/>
+      <c r="BO33" s="6"/>
+      <c r="BP33" s="11"/>
+      <c r="BQ33" s="11"/>
+      <c r="BR33" s="11"/>
+      <c r="BS33" s="6"/>
+      <c r="BT33" s="6"/>
+      <c r="BU33" s="11"/>
+      <c r="BV33" s="11"/>
+      <c r="BW33" s="11"/>
+      <c r="BX33" s="6"/>
+      <c r="BY33" s="6"/>
+      <c r="BZ33" s="11"/>
+      <c r="CA33" s="11"/>
+      <c r="CB33" s="11"/>
+      <c r="CC33" s="6"/>
+      <c r="CD33" s="6"/>
+      <c r="CE33" s="11"/>
+      <c r="CF33" s="11"/>
+      <c r="CG33" s="11"/>
+      <c r="CH33" s="6"/>
+      <c r="CI33" s="6"/>
+      <c r="CJ33" s="11"/>
+      <c r="CK33" s="11"/>
+      <c r="CL33" s="11"/>
+      <c r="CM33" s="11"/>
+      <c r="CN33" s="7"/>
+      <c r="CO33" s="7"/>
+      <c r="CP33" s="11"/>
+      <c r="CQ33" s="11"/>
+      <c r="CR33" s="11"/>
+      <c r="CS33" s="11"/>
+      <c r="CT33" s="6"/>
+      <c r="CU33" s="6"/>
+      <c r="CV33" s="11"/>
+      <c r="CW33" s="11"/>
+      <c r="CX33" s="11"/>
+      <c r="CY33" s="11"/>
+      <c r="CZ33" s="6"/>
+      <c r="DA33" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>